<commit_message>
Add Excel dropdown validation for price list template.
Template now includes service and promo picklists from the catalog sheet, with formulas that auto-fill specialty and service code.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/downloads/price-list-template.xlsx
+++ b/public/downloads/price-list-template.xlsx
@@ -185,6 +185,29 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B300">
+      <formula1>'Справочник услуг'!$B$2:$B$42</formula1>
+      <promptTitle>Услуга</promptTitle>
+      <prompt>Выберите услугу из справочника. Специализация и код заполнятся автоматически.</prompt>
+      <errorTitle>Недопустимое значение</errorTitle>
+      <error>Выберите значение из списка справочника.</error>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C300">
+      <formula1>'Справочник услуг'!$C$2:$C$42</formula1>
+      <promptTitle>Код услуги</promptTitle>
+      <prompt>Или выберите код услуги из справочника.</prompt>
+      <errorTitle>Недопустимое значение</errorTitle>
+      <error>Выберите значение из списка справочника.</error>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F300">
+      <formula1>"да,нет"</formula1>
+      <promptTitle>Акция</promptTitle>
+      <prompt>Укажите «да» или «нет».</prompt>
+      <errorTitle>Недопустимое значение</errorTitle>
+      <error>Выберите значение из списка справочника.</error>
+    </dataValidation>
+  </dataValidations>
   <legacyDrawing r:id="rId_comments_vml1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix Excel dropdown lists using workbook defined names.
Excel ignores cross-sheet list validation without named ranges. Apply picklists to template and export, and replace zip entries safely.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/downloads/price-list-template.xlsx
+++ b/public/downloads/price-list-template.xlsx
@@ -5,6 +5,9 @@
     <sheet name="Прайс" sheetId="1" r:id="rIdSheet1" state="visible"/>
     <sheet name="Справочник услуг" sheetId="2" r:id="rIdSheet2" state="visible"/>
   </sheets>
+  <definedNames>
+    <definedName name="StClinikServices">'Справочник услуг'!$B$2:$B$42</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -185,18 +188,11 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B300">
-      <formula1>'Справочник услуг'!$B$2:$B$42</formula1>
+      <formula1>StClinikServices</formula1>
       <promptTitle>Услуга</promptTitle>
-      <prompt>Выберите услугу из справочника. Специализация и код заполнятся автоматически.</prompt>
-      <errorTitle>Недопустимое значение</errorTitle>
-      <error>Выберите значение из списка справочника.</error>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C300">
-      <formula1>'Справочник услуг'!$C$2:$C$42</formula1>
-      <promptTitle>Код услуги</promptTitle>
-      <prompt>Или выберите код услуги из справочника.</prompt>
+      <prompt>Выберите услугу из справочника. Специализация и код подставятся автоматически.</prompt>
       <errorTitle>Недопустимое значение</errorTitle>
       <error>Выберите значение из списка справочника.</error>
     </dataValidation>

</xml_diff>